<commit_message>
network charges pricing model
</commit_message>
<xml_diff>
--- a/inst/ext_data/scenario_parameters.xlsx
+++ b/inst/ext_data/scenario_parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joe\pkgs\depmicrosimr\inst\ext_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989D9BBD-DEA7-415A-ABC8-D59A854C0990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5160988-B94B-4C14-90C5-A6FCA9804B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="124">
   <si>
     <t>category</t>
   </si>
@@ -326,11 +326,116 @@
   <si>
     <t>handling negative prices</t>
   </si>
+  <si>
+    <t>technical</t>
+  </si>
+  <si>
+    <t>minimum household hourly flexibility</t>
+  </si>
+  <si>
+    <t>maximum household hourly flexibility</t>
+  </si>
+  <si>
+    <t>min_flex</t>
+  </si>
+  <si>
+    <t>max_flex</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>hourly MAD assuming 2026 dynamic prices and LP1 load</t>
+  </si>
+  <si>
+    <t>max risk aversion</t>
+  </si>
+  <si>
+    <t>theta.</t>
+  </si>
+  <si>
+    <t>dynamic price cap scale</t>
+  </si>
+  <si>
+    <t>dynamic_price_cap_scale</t>
+  </si>
+  <si>
+    <t>the current cap is dynamic_price_cap_scale*current flat price</t>
+  </si>
+  <si>
+    <t>night network charge</t>
+  </si>
+  <si>
+    <t>peak network charge</t>
+  </si>
+  <si>
+    <t>polixy</t>
+  </si>
+  <si>
+    <t>vat rate electricity</t>
+  </si>
+  <si>
+    <t>vat_rate</t>
+  </si>
+  <si>
+    <t>day network charge</t>
+  </si>
+  <si>
+    <t>day_network_charge_2020</t>
+  </si>
+  <si>
+    <t>night_network_charge_2020</t>
+  </si>
+  <si>
+    <t>peak_network_charge_2020</t>
+  </si>
+  <si>
+    <t>day_network_charge_2030</t>
+  </si>
+  <si>
+    <t>night_network_charge_2030</t>
+  </si>
+  <si>
+    <t>peak_network_charge_2030</t>
+  </si>
+  <si>
+    <t>regulated grid charges+supplier uplift (costs, margin)</t>
+  </si>
+  <si>
+    <t>15% below 2026 values</t>
+  </si>
+  <si>
+    <t>10% above 2026 values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30% above </t>
+  </si>
+  <si>
+    <t>day_network_charge_2026</t>
+  </si>
+  <si>
+    <t>night_network_charge_2026</t>
+  </si>
+  <si>
+    <t>peak_network_charge_2026</t>
+  </si>
+  <si>
+    <t>day_network_charge_2040</t>
+  </si>
+  <si>
+    <t>night_network_charge_2040</t>
+  </si>
+  <si>
+    <t>peak_network_charge_2040</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -393,12 +498,30 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dotted">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dotted">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -407,7 +530,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -424,6 +547,13 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="2" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -832,7 +962,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C8E1679-ADB0-42D7-8103-5D0EB0C9F50E}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -897,253 +1027,249 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>104</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>105</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>63</v>
+        <v>106</v>
       </c>
       <c r="D4">
-        <v>0.4</v>
-      </c>
-      <c r="E4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="1"/>
+        <v>0.09</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5">
-        <v>0.4</v>
+      <c r="A5" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D5" s="8">
+        <v>0.16838500000000001</v>
       </c>
       <c r="E5" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="1"/>
+      <c r="F5" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6">
-        <v>0.52500000000000002</v>
+      <c r="A6" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="D6" s="8">
+        <v>7.2419999999999998E-2</v>
       </c>
       <c r="E6" t="s">
-        <v>65</v>
-      </c>
-      <c r="F6" s="1"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="D7">
-        <v>0.52500000000000002</v>
+      <c r="A7" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="8">
+        <v>0.19167500000000001</v>
       </c>
       <c r="E7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F7" s="1"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" t="s">
-        <v>46</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>71</v>
+      <c r="A8" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>118</v>
       </c>
       <c r="D8">
-        <v>0.52500000000000002</v>
+        <v>0.1981</v>
       </c>
       <c r="E8" t="s">
-        <v>65</v>
-      </c>
-      <c r="F8" s="1"/>
+        <v>41</v>
+      </c>
+      <c r="F8" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B9" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>67</v>
+      <c r="A9" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>119</v>
       </c>
       <c r="D9">
-        <v>1.0880000000000001</v>
+        <v>8.5199999999999998E-2</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="1"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>68</v>
+      <c r="A10" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>120</v>
       </c>
       <c r="D10">
-        <v>1.0880000000000001</v>
+        <v>0.22550000000000001</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
-      </c>
-      <c r="F10" s="1"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11">
-        <v>1.0880000000000001</v>
+      <c r="A11" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="8">
+        <v>0.21791000000000002</v>
       </c>
       <c r="E11" t="s">
-        <v>65</v>
-      </c>
-      <c r="F11" s="1"/>
+        <v>41</v>
+      </c>
+      <c r="F11" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="D12">
-        <v>1.0660000000000001</v>
+      <c r="A12" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="D12" s="8">
+        <v>9.3720000000000012E-2</v>
       </c>
       <c r="E12" t="s">
-        <v>65</v>
-      </c>
-      <c r="F12" s="1"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D13">
-        <v>1.0660000000000001</v>
+      <c r="A13" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" s="8">
+        <v>0.24805000000000002</v>
       </c>
       <c r="E13" t="s">
-        <v>65</v>
-      </c>
-      <c r="F13" s="1"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="D14">
-        <v>1.0660000000000001</v>
+      <c r="A14" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D14" s="8">
+        <v>0.25752999999999998</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
-      </c>
-      <c r="F14" s="1"/>
+        <v>41</v>
+      </c>
+      <c r="F14" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D15">
-        <v>3.1</v>
+      <c r="A15" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" s="8">
+        <v>0.11076</v>
       </c>
       <c r="E15" t="s">
-        <v>65</v>
-      </c>
-      <c r="F15" s="1"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>38</v>
-      </c>
-      <c r="B16" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16">
-        <v>3.1</v>
+      <c r="A16" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="D16" s="8">
+        <v>0.29315000000000002</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
-      </c>
-      <c r="F16" s="1"/>
+        <v>41</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>38</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="D17">
-        <v>3.1</v>
+        <v>0.4</v>
       </c>
       <c r="E17" t="s">
-        <v>65</v>
+        <v>41</v>
       </c>
       <c r="F17" s="1"/>
     </row>
@@ -1152,31 +1278,34 @@
         <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="D18">
-        <v>130</v>
+        <v>0.4</v>
       </c>
       <c r="E18" t="s">
-        <v>77</v>
+        <v>41</v>
       </c>
       <c r="F18" s="1"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="D19">
-        <v>215</v>
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="E19" t="s">
+        <v>65</v>
       </c>
       <c r="F19" s="1"/>
     </row>
@@ -1185,13 +1314,16 @@
         <v>38</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>45</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="D20">
-        <v>265</v>
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="E20" t="s">
+        <v>65</v>
       </c>
       <c r="F20" s="1"/>
     </row>
@@ -1200,13 +1332,16 @@
         <v>38</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D21">
-        <v>320</v>
+        <v>0.52500000000000002</v>
+      </c>
+      <c r="E21" t="s">
+        <v>65</v>
       </c>
       <c r="F21" s="1"/>
     </row>
@@ -1215,88 +1350,387 @@
         <v>38</v>
       </c>
       <c r="B22" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="D22">
-        <v>350</v>
+        <v>1.0880000000000001</v>
+      </c>
+      <c r="E22" t="s">
+        <v>65</v>
       </c>
       <c r="F22" s="1"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>14</v>
+        <v>47</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>68</v>
       </c>
       <c r="D23">
-        <v>0.594322503</v>
+        <v>1.0880000000000001</v>
       </c>
       <c r="E23" t="s">
-        <v>15</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="F23" s="1"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="B24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>8</v>
+        <v>48</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D24">
-        <v>4.8274562E-2</v>
+        <v>1.0880000000000001</v>
       </c>
       <c r="E24" t="s">
-        <v>15</v>
-      </c>
-      <c r="F24" t="s">
-        <v>62</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="F24" s="1"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="B25" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>17</v>
+        <v>59</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>60</v>
       </c>
       <c r="D25">
-        <v>0.03</v>
+        <v>1.0660000000000001</v>
       </c>
       <c r="E25" t="s">
-        <v>18</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="F25" s="1"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26">
+        <v>1.0660000000000001</v>
+      </c>
+      <c r="E26" t="s">
+        <v>65</v>
+      </c>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D27">
+        <v>1.0660000000000001</v>
+      </c>
+      <c r="E27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F27" s="1"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D28">
+        <v>3.1</v>
+      </c>
+      <c r="E28" t="s">
+        <v>65</v>
+      </c>
+      <c r="F28" s="1"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B29" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D29">
+        <v>3.1</v>
+      </c>
+      <c r="E29" t="s">
+        <v>65</v>
+      </c>
+      <c r="F29" s="1"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D30">
+        <v>3.1</v>
+      </c>
+      <c r="E30" t="s">
+        <v>65</v>
+      </c>
+      <c r="F30" s="1"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" t="s">
+        <v>99</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31" t="s">
+        <v>65</v>
+      </c>
+      <c r="F31" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32">
+        <v>130</v>
+      </c>
+      <c r="E32" t="s">
+        <v>77</v>
+      </c>
+      <c r="F32" s="1"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" t="s">
+        <v>82</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33">
+        <v>215</v>
+      </c>
+      <c r="F33" s="1"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34" t="s">
+        <v>83</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34">
+        <v>265</v>
+      </c>
+      <c r="F34" s="1"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" t="s">
+        <v>84</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35">
+        <v>320</v>
+      </c>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" t="s">
+        <v>85</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D36">
+        <v>350</v>
+      </c>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>90</v>
+      </c>
+      <c r="B37" t="s">
+        <v>91</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D37">
+        <v>2</v>
+      </c>
+      <c r="E37" t="s">
+        <v>95</v>
+      </c>
+      <c r="F37" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>90</v>
+      </c>
+      <c r="B38" t="s">
+        <v>92</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D38">
+        <v>30</v>
+      </c>
+      <c r="E38" t="s">
+        <v>95</v>
+      </c>
+      <c r="F38" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>7</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39">
+        <v>0.594322503</v>
+      </c>
+      <c r="E39" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>7</v>
+      </c>
+      <c r="B40" t="s">
+        <v>61</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40">
+        <v>4.8274562E-2</v>
+      </c>
+      <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" t="s">
+        <v>6</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41">
+        <v>0.03</v>
+      </c>
+      <c r="E41" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" t="s">
         <v>86</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C42" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D26">
+      <c r="D42">
         <v>10</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E42" t="s">
         <v>87</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F42" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" t="s">
+        <v>97</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D43">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>